<commit_message>
Unique team big board logic added, team needs generated on current roster and variable weights, UI changes (previoius selections, team needs, big board changes), fixed bug where you could sim to already completed rounds
</commit_message>
<xml_diff>
--- a/Files/TestFiles/PositionNeeds.xlsx
+++ b/Files/TestFiles/PositionNeeds.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Important Files/Madden 25/DraftTool/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Git/MaddenDraftTool/Files/TestFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="128" documentId="8_{7C439BFB-0DBF-4097-AD0B-C529E75DCE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE98DD73-D4ED-43DE-86AC-4ADC36BD34BF}"/>
+  <xr:revisionPtr revIDLastSave="205" documentId="8_{7C439BFB-0DBF-4097-AD0B-C529E75DCE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02AB542E-737A-4514-9D37-899FAADDCD40}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE15C3C6-B90C-4AA8-AF55-EC28F49C3043}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="TierNeedLogic" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">TierNeedLogic!$A$1:$H$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">TierNeedLogic!$A$1:$H$87</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="80">
   <si>
     <t>QB</t>
   </si>
@@ -270,6 +270,15 @@
   </si>
   <si>
     <t>DT4</t>
+  </si>
+  <si>
+    <t>QB1</t>
+  </si>
+  <si>
+    <t>FB</t>
+  </si>
+  <si>
+    <t>FB1</t>
   </si>
 </sst>
 </file>
@@ -328,6 +337,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -647,7 +660,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB6437B3-F8C6-4C30-BAA1-BB8B4D93E54D}">
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
@@ -691,25 +704,25 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="F2">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="G2">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="H2">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -723,42 +736,42 @@
         <v>29</v>
       </c>
       <c r="D3">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>59</v>
+      </c>
+      <c r="G3">
         <v>60</v>
       </c>
-      <c r="F3">
-        <v>64</v>
-      </c>
-      <c r="G3">
-        <v>65</v>
-      </c>
       <c r="H3">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F4">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="G4">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="H4">
         <v>99</v>
@@ -775,16 +788,16 @@
         <v>30</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>74</v>
+      </c>
+      <c r="G5">
         <v>75</v>
-      </c>
-      <c r="F5">
-        <v>79</v>
-      </c>
-      <c r="G5">
-        <v>80</v>
       </c>
       <c r="H5">
         <v>99</v>
@@ -795,25 +808,25 @@
         <v>1</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D6">
         <v>2</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F6">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="G6">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="H6">
-        <v>77</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -827,19 +840,19 @@
         <v>31</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>69</v>
+      </c>
+      <c r="G7">
         <v>70</v>
       </c>
-      <c r="F7">
-        <v>72</v>
-      </c>
-      <c r="G7">
-        <v>73</v>
-      </c>
       <c r="H7">
-        <v>77</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -847,48 +860,48 @@
         <v>1</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>74</v>
+        <v>31</v>
       </c>
       <c r="D8">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F8">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="G8">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="H8">
-        <v>70</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>74</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
       <c r="F9">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="G9">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="H9">
         <v>99</v>
@@ -905,16 +918,16 @@
         <v>32</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>74</v>
+      </c>
+      <c r="G10">
         <v>75</v>
-      </c>
-      <c r="F10">
-        <v>79</v>
-      </c>
-      <c r="G10">
-        <v>80</v>
       </c>
       <c r="H10">
         <v>99</v>
@@ -925,25 +938,25 @@
         <v>2</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F11">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G11">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H11">
-        <v>82</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -957,19 +970,19 @@
         <v>33</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>74</v>
+      </c>
+      <c r="G12">
         <v>75</v>
       </c>
-      <c r="F12">
-        <v>77</v>
-      </c>
-      <c r="G12">
-        <v>78</v>
-      </c>
       <c r="H12">
-        <v>82</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -977,25 +990,25 @@
         <v>2</v>
       </c>
       <c r="B13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D13">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F13">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="G13">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="H13">
-        <v>79</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1009,19 +1022,19 @@
         <v>34</v>
       </c>
       <c r="D14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>69</v>
+      </c>
+      <c r="G14">
         <v>70</v>
       </c>
-      <c r="F14">
-        <v>73</v>
-      </c>
-      <c r="G14">
-        <v>74</v>
-      </c>
       <c r="H14">
-        <v>79</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -1029,25 +1042,25 @@
         <v>2</v>
       </c>
       <c r="B15">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F15">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="G15">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="H15">
-        <v>74</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -1064,16 +1077,16 @@
         <v>1</v>
       </c>
       <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>67</v>
+      </c>
+      <c r="G16">
         <v>68</v>
       </c>
-      <c r="F16">
-        <v>71</v>
-      </c>
-      <c r="G16">
-        <v>72</v>
-      </c>
       <c r="H16">
-        <v>74</v>
+        <v>99</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1081,48 +1094,48 @@
         <v>2</v>
       </c>
       <c r="B17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>73</v>
+        <v>35</v>
       </c>
       <c r="D17">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="F17">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="G17">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="H17">
-        <v>70</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B18">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="D18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E18">
         <v>0</v>
       </c>
       <c r="F18">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G18">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H18">
         <v>99</v>
@@ -1139,19 +1152,19 @@
         <v>36</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>69</v>
+      </c>
+      <c r="G19">
         <v>70</v>
       </c>
-      <c r="F19">
-        <v>74</v>
-      </c>
-      <c r="G19">
-        <v>75</v>
-      </c>
       <c r="H19">
-        <v>85</v>
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1159,25 +1172,25 @@
         <v>3</v>
       </c>
       <c r="B20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D20">
         <v>2</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F20">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G20">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="H20">
-        <v>72</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -1191,19 +1204,19 @@
         <v>37</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>64</v>
+      </c>
+      <c r="G21">
         <v>65</v>
       </c>
-      <c r="F21">
-        <v>66</v>
-      </c>
-      <c r="G21">
-        <v>67</v>
-      </c>
       <c r="H21">
-        <v>72</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1211,48 +1224,48 @@
         <v>3</v>
       </c>
       <c r="B22">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C22" t="s">
-        <v>75</v>
+        <v>37</v>
       </c>
       <c r="D22">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="F22">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G22">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H22">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B23">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C23" t="s">
-        <v>38</v>
+        <v>75</v>
       </c>
       <c r="D23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E23">
         <v>0</v>
       </c>
       <c r="F23">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G23">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H23">
         <v>99</v>
@@ -1269,16 +1282,16 @@
         <v>38</v>
       </c>
       <c r="D24">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E24">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="F24">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G24">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H24">
         <v>99</v>
@@ -1289,25 +1302,25 @@
         <v>4</v>
       </c>
       <c r="B25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D25">
         <v>2</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="F25">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="G25">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="H25">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -1321,42 +1334,42 @@
         <v>39</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>62</v>
+      </c>
+      <c r="G26">
         <v>63</v>
       </c>
-      <c r="F26">
-        <v>64</v>
-      </c>
-      <c r="G26">
-        <v>65</v>
-      </c>
       <c r="H26">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="F27">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G27">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H27">
         <v>99</v>
@@ -1373,16 +1386,16 @@
         <v>40</v>
       </c>
       <c r="D28">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E28">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="F28">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G28">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H28">
         <v>99</v>
@@ -1393,25 +1406,25 @@
         <v>5</v>
       </c>
       <c r="B29">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D29">
         <v>2</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="F29">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="G29">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="H29">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -1425,42 +1438,42 @@
         <v>41</v>
       </c>
       <c r="D30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E30">
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <v>62</v>
+      </c>
+      <c r="G30">
         <v>63</v>
       </c>
-      <c r="F30">
-        <v>64</v>
-      </c>
-      <c r="G30">
-        <v>65</v>
-      </c>
       <c r="H30">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="F31">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G31">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H31">
         <v>99</v>
@@ -1477,16 +1490,16 @@
         <v>42</v>
       </c>
       <c r="D32">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E32">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="F32">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G32">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H32">
         <v>99</v>
@@ -1497,25 +1510,25 @@
         <v>6</v>
       </c>
       <c r="B33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D33">
         <v>2</v>
       </c>
       <c r="E33">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="F33">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="G33">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="H33">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -1529,42 +1542,42 @@
         <v>43</v>
       </c>
       <c r="D34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E34">
+        <v>0</v>
+      </c>
+      <c r="F34">
+        <v>62</v>
+      </c>
+      <c r="G34">
         <v>63</v>
       </c>
-      <c r="F34">
-        <v>64</v>
-      </c>
-      <c r="G34">
-        <v>65</v>
-      </c>
       <c r="H34">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C35" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D35">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E35">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="F35">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G35">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H35">
         <v>99</v>
@@ -1581,16 +1594,16 @@
         <v>44</v>
       </c>
       <c r="D36">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E36">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="F36">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G36">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H36">
         <v>99</v>
@@ -1601,25 +1614,25 @@
         <v>7</v>
       </c>
       <c r="B37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D37">
         <v>2</v>
       </c>
       <c r="E37">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="F37">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="G37">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="H37">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
@@ -1633,42 +1646,42 @@
         <v>45</v>
       </c>
       <c r="D38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E38">
+        <v>0</v>
+      </c>
+      <c r="F38">
+        <v>62</v>
+      </c>
+      <c r="G38">
         <v>63</v>
       </c>
-      <c r="F38">
-        <v>64</v>
-      </c>
-      <c r="G38">
-        <v>65</v>
-      </c>
       <c r="H38">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B39">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D39">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="F39">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G39">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H39">
         <v>99</v>
@@ -1685,16 +1698,16 @@
         <v>46</v>
       </c>
       <c r="D40">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E40">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="F40">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G40">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H40">
         <v>99</v>
@@ -1705,25 +1718,25 @@
         <v>8</v>
       </c>
       <c r="B41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D41">
         <v>2</v>
       </c>
       <c r="E41">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="F41">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="G41">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="H41">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -1737,42 +1750,42 @@
         <v>47</v>
       </c>
       <c r="D42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E42">
+        <v>0</v>
+      </c>
+      <c r="F42">
+        <v>62</v>
+      </c>
+      <c r="G42">
         <v>63</v>
       </c>
-      <c r="F42">
-        <v>64</v>
-      </c>
-      <c r="G42">
-        <v>65</v>
-      </c>
       <c r="H42">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C43" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E43">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="F43">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="G43">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H43">
         <v>99</v>
@@ -1789,19 +1802,19 @@
         <v>48</v>
       </c>
       <c r="D44">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E44">
+        <v>0</v>
+      </c>
+      <c r="F44">
+        <v>69</v>
+      </c>
+      <c r="G44">
         <v>70</v>
       </c>
-      <c r="F44">
-        <v>74</v>
-      </c>
-      <c r="G44">
-        <v>75</v>
-      </c>
       <c r="H44">
-        <v>89</v>
+        <v>99</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -1809,25 +1822,25 @@
         <v>9</v>
       </c>
       <c r="B45">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D45">
         <v>2</v>
       </c>
       <c r="E45">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F45">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G45">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="H45">
-        <v>75</v>
+        <v>99</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -1841,42 +1854,42 @@
         <v>49</v>
       </c>
       <c r="D46">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E46">
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>64</v>
+      </c>
+      <c r="G46">
         <v>65</v>
       </c>
-      <c r="F46">
-        <v>67</v>
-      </c>
-      <c r="G46">
-        <v>68</v>
-      </c>
       <c r="H46">
-        <v>75</v>
+        <v>99</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B47">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C47" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D47">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E47">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="F47">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G47">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H47">
         <v>99</v>
@@ -1893,19 +1906,19 @@
         <v>50</v>
       </c>
       <c r="D48">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E48">
+        <v>0</v>
+      </c>
+      <c r="F48">
+        <v>69</v>
+      </c>
+      <c r="G48">
         <v>70</v>
       </c>
-      <c r="F48">
-        <v>74</v>
-      </c>
-      <c r="G48">
-        <v>75</v>
-      </c>
       <c r="H48">
-        <v>89</v>
+        <v>99</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
@@ -1913,25 +1926,25 @@
         <v>10</v>
       </c>
       <c r="B49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C49" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D49">
         <v>2</v>
       </c>
       <c r="E49">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F49">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="G49">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="H49">
-        <v>75</v>
+        <v>99</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
@@ -1945,42 +1958,42 @@
         <v>51</v>
       </c>
       <c r="D50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E50">
+        <v>0</v>
+      </c>
+      <c r="F50">
+        <v>64</v>
+      </c>
+      <c r="G50">
         <v>65</v>
       </c>
-      <c r="F50">
-        <v>67</v>
-      </c>
-      <c r="G50">
-        <v>68</v>
-      </c>
       <c r="H50">
-        <v>75</v>
+        <v>99</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C51" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D51">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E51">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="F51">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G51">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H51">
         <v>99</v>
@@ -1997,16 +2010,16 @@
         <v>52</v>
       </c>
       <c r="D52">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E52">
+        <v>0</v>
+      </c>
+      <c r="F52">
+        <v>69</v>
+      </c>
+      <c r="G52">
         <v>70</v>
-      </c>
-      <c r="F52">
-        <v>77</v>
-      </c>
-      <c r="G52">
-        <v>78</v>
       </c>
       <c r="H52">
         <v>99</v>
@@ -2017,25 +2030,25 @@
         <v>11</v>
       </c>
       <c r="B53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C53" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D53">
         <v>2</v>
       </c>
       <c r="E53">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F53">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="G53">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="H53">
-        <v>85</v>
+        <v>99</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
@@ -2049,19 +2062,19 @@
         <v>53</v>
       </c>
       <c r="D54">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E54">
+        <v>0</v>
+      </c>
+      <c r="F54">
+        <v>69</v>
+      </c>
+      <c r="G54">
         <v>70</v>
       </c>
-      <c r="F54">
-        <v>74</v>
-      </c>
-      <c r="G54">
-        <v>75</v>
-      </c>
       <c r="H54">
-        <v>80</v>
+        <v>99</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
@@ -2069,25 +2082,25 @@
         <v>11</v>
       </c>
       <c r="B55">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C55" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D55">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E55">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F55">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="G55">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="H55">
-        <v>75</v>
+        <v>99</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
@@ -2101,19 +2114,19 @@
         <v>54</v>
       </c>
       <c r="D56">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E56">
+        <v>0</v>
+      </c>
+      <c r="F56">
+        <v>69</v>
+      </c>
+      <c r="G56">
         <v>70</v>
       </c>
-      <c r="F56">
-        <v>72</v>
-      </c>
-      <c r="G56">
-        <v>73</v>
-      </c>
       <c r="H56">
-        <v>75</v>
+        <v>99</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
@@ -2121,39 +2134,39 @@
         <v>11</v>
       </c>
       <c r="B57">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C57" t="s">
-        <v>76</v>
+        <v>54</v>
       </c>
       <c r="D57">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E57">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F57">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="G57">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="H57">
-        <v>69</v>
+        <v>99</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B58">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C58" t="s">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="D58">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E58">
         <v>0</v>
@@ -2179,16 +2192,16 @@
         <v>55</v>
       </c>
       <c r="D59">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E59">
+        <v>0</v>
+      </c>
+      <c r="F59">
+        <v>64</v>
+      </c>
+      <c r="G59">
         <v>65</v>
-      </c>
-      <c r="F59">
-        <v>74</v>
-      </c>
-      <c r="G59">
-        <v>75</v>
       </c>
       <c r="H59">
         <v>99</v>
@@ -2199,48 +2212,48 @@
         <v>12</v>
       </c>
       <c r="B60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C60" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E60">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="F60">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="G60">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="H60">
-        <v>72</v>
+        <v>99</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B61">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C61" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D61">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E61">
         <v>0</v>
       </c>
       <c r="F61">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="G61">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H61">
         <v>99</v>
@@ -2257,16 +2270,16 @@
         <v>57</v>
       </c>
       <c r="D62">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E62">
+        <v>0</v>
+      </c>
+      <c r="F62">
+        <v>64</v>
+      </c>
+      <c r="G62">
         <v>65</v>
-      </c>
-      <c r="F62">
-        <v>74</v>
-      </c>
-      <c r="G62">
-        <v>75</v>
       </c>
       <c r="H62">
         <v>99</v>
@@ -2277,48 +2290,48 @@
         <v>13</v>
       </c>
       <c r="B63">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C63" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D63">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E63">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="F63">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="G63">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="H63">
-        <v>72</v>
+        <v>99</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B64">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C64" t="s">
+        <v>58</v>
+      </c>
+      <c r="D64">
+        <v>1</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+      <c r="F64">
         <v>59</v>
       </c>
-      <c r="D64">
-        <v>2</v>
-      </c>
-      <c r="E64">
-        <v>0</v>
-      </c>
-      <c r="F64">
-        <v>64</v>
-      </c>
       <c r="G64">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="H64">
         <v>99</v>
@@ -2335,16 +2348,16 @@
         <v>59</v>
       </c>
       <c r="D65">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>64</v>
+      </c>
+      <c r="G65">
         <v>65</v>
-      </c>
-      <c r="F65">
-        <v>74</v>
-      </c>
-      <c r="G65">
-        <v>75</v>
       </c>
       <c r="H65">
         <v>99</v>
@@ -2355,48 +2368,48 @@
         <v>14</v>
       </c>
       <c r="B66">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C66" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D66">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E66">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="F66">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="G66">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="H66">
-        <v>72</v>
+        <v>99</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C67" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D67">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E67">
         <v>0</v>
       </c>
       <c r="F67">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="G67">
-        <v>75</v>
+        <v>63</v>
       </c>
       <c r="H67">
         <v>99</v>
@@ -2413,16 +2426,16 @@
         <v>61</v>
       </c>
       <c r="D68">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E68">
+        <v>0</v>
+      </c>
+      <c r="F68">
+        <v>74</v>
+      </c>
+      <c r="G68">
         <v>75</v>
-      </c>
-      <c r="F68">
-        <v>79</v>
-      </c>
-      <c r="G68">
-        <v>80</v>
       </c>
       <c r="H68">
         <v>99</v>
@@ -2433,25 +2446,25 @@
         <v>15</v>
       </c>
       <c r="B69">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C69" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D69">
         <v>2</v>
       </c>
       <c r="E69">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F69">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="G69">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H69">
-        <v>82</v>
+        <v>99</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
@@ -2465,19 +2478,19 @@
         <v>62</v>
       </c>
       <c r="D70">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E70">
+        <v>0</v>
+      </c>
+      <c r="F70">
+        <v>74</v>
+      </c>
+      <c r="G70">
         <v>75</v>
       </c>
-      <c r="F70">
-        <v>77</v>
-      </c>
-      <c r="G70">
-        <v>78</v>
-      </c>
       <c r="H70">
-        <v>82</v>
+        <v>99</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
@@ -2485,25 +2498,25 @@
         <v>15</v>
       </c>
       <c r="B71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C71" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D71">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E71">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F71">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="G71">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="H71">
-        <v>79</v>
+        <v>99</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
@@ -2517,19 +2530,19 @@
         <v>63</v>
       </c>
       <c r="D72">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E72">
+        <v>0</v>
+      </c>
+      <c r="F72">
+        <v>69</v>
+      </c>
+      <c r="G72">
         <v>70</v>
       </c>
-      <c r="F72">
-        <v>73</v>
-      </c>
-      <c r="G72">
-        <v>74</v>
-      </c>
       <c r="H72">
-        <v>79</v>
+        <v>99</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
@@ -2537,25 +2550,25 @@
         <v>15</v>
       </c>
       <c r="B73">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C73" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E73">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F73">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="G73">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="H73">
-        <v>74</v>
+        <v>99</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
@@ -2572,16 +2585,16 @@
         <v>1</v>
       </c>
       <c r="E74">
+        <v>0</v>
+      </c>
+      <c r="F74">
+        <v>67</v>
+      </c>
+      <c r="G74">
         <v>68</v>
       </c>
-      <c r="F74">
-        <v>71</v>
-      </c>
-      <c r="G74">
-        <v>72</v>
-      </c>
       <c r="H74">
-        <v>74</v>
+        <v>99</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
@@ -2589,48 +2602,48 @@
         <v>15</v>
       </c>
       <c r="B75">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C75" t="s">
+        <v>64</v>
+      </c>
+      <c r="D75">
+        <v>1</v>
+      </c>
+      <c r="E75">
+        <v>68</v>
+      </c>
+      <c r="F75">
+        <v>71</v>
+      </c>
+      <c r="G75">
         <v>72</v>
       </c>
-      <c r="D75">
-        <v>0.5</v>
-      </c>
-      <c r="E75">
-        <v>0</v>
-      </c>
-      <c r="F75">
-        <v>64</v>
-      </c>
-      <c r="G75">
-        <v>65</v>
-      </c>
       <c r="H75">
-        <v>70</v>
+        <v>99</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B76">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C76" t="s">
+        <v>72</v>
+      </c>
+      <c r="D76">
+        <v>1</v>
+      </c>
+      <c r="E76">
+        <v>0</v>
+      </c>
+      <c r="F76">
+        <v>64</v>
+      </c>
+      <c r="G76">
         <v>65</v>
-      </c>
-      <c r="D76">
-        <v>2</v>
-      </c>
-      <c r="E76">
-        <v>0</v>
-      </c>
-      <c r="F76">
-        <v>69</v>
-      </c>
-      <c r="G76">
-        <v>70</v>
       </c>
       <c r="H76">
         <v>99</v>
@@ -2647,16 +2660,16 @@
         <v>65</v>
       </c>
       <c r="D77">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E77">
+        <v>0</v>
+      </c>
+      <c r="F77">
+        <v>69</v>
+      </c>
+      <c r="G77">
         <v>70</v>
-      </c>
-      <c r="F77">
-        <v>75</v>
-      </c>
-      <c r="G77">
-        <v>76</v>
       </c>
       <c r="H77">
         <v>99</v>
@@ -2667,25 +2680,25 @@
         <v>16</v>
       </c>
       <c r="B78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C78" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D78">
         <v>2</v>
       </c>
       <c r="E78">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F78">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="G78">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="H78">
-        <v>75</v>
+        <v>99</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
@@ -2699,42 +2712,42 @@
         <v>66</v>
       </c>
       <c r="D79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E79">
+        <v>0</v>
+      </c>
+      <c r="F79">
+        <v>65</v>
+      </c>
+      <c r="G79">
         <v>66</v>
       </c>
-      <c r="F79">
-        <v>67</v>
-      </c>
-      <c r="G79">
-        <v>68</v>
-      </c>
       <c r="H79">
-        <v>75</v>
+        <v>99</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C80" t="s">
+        <v>66</v>
+      </c>
+      <c r="D80">
+        <v>1</v>
+      </c>
+      <c r="E80">
+        <v>66</v>
+      </c>
+      <c r="F80">
         <v>67</v>
       </c>
-      <c r="D80">
-        <v>2</v>
-      </c>
-      <c r="E80">
-        <v>0</v>
-      </c>
-      <c r="F80">
-        <v>69</v>
-      </c>
       <c r="G80">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H80">
         <v>99</v>
@@ -2751,16 +2764,16 @@
         <v>67</v>
       </c>
       <c r="D81">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E81">
+        <v>0</v>
+      </c>
+      <c r="F81">
+        <v>69</v>
+      </c>
+      <c r="G81">
         <v>70</v>
-      </c>
-      <c r="F81">
-        <v>75</v>
-      </c>
-      <c r="G81">
-        <v>76</v>
       </c>
       <c r="H81">
         <v>99</v>
@@ -2771,25 +2784,25 @@
         <v>17</v>
       </c>
       <c r="B82">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C82" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D82">
         <v>2</v>
       </c>
       <c r="E82">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F82">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="G82">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="H82">
-        <v>75</v>
+        <v>99</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
@@ -2803,39 +2816,39 @@
         <v>68</v>
       </c>
       <c r="D83">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E83">
+        <v>0</v>
+      </c>
+      <c r="F83">
+        <v>65</v>
+      </c>
+      <c r="G83">
         <v>66</v>
       </c>
-      <c r="F83">
-        <v>67</v>
-      </c>
-      <c r="G83">
-        <v>68</v>
-      </c>
       <c r="H83">
-        <v>75</v>
+        <v>99</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B84">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C84" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D84">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="E84">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="F84">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G84">
         <v>68</v>
@@ -2846,16 +2859,16 @@
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B85">
         <v>1</v>
       </c>
       <c r="C85" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D85">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E85">
         <v>0</v>
@@ -2872,32 +2885,84 @@
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>19</v>
+      </c>
+      <c r="B86">
+        <v>1</v>
+      </c>
+      <c r="C86" t="s">
+        <v>70</v>
+      </c>
+      <c r="D86">
+        <v>2</v>
+      </c>
+      <c r="E86">
+        <v>0</v>
+      </c>
+      <c r="F86">
+        <v>69</v>
+      </c>
+      <c r="G86">
+        <v>68</v>
+      </c>
+      <c r="H86">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>27</v>
       </c>
-      <c r="B86">
-        <v>1</v>
-      </c>
-      <c r="C86" t="s">
+      <c r="B87">
+        <v>1</v>
+      </c>
+      <c r="C87" t="s">
         <v>28</v>
       </c>
-      <c r="D86">
-        <v>1.5</v>
-      </c>
-      <c r="E86">
-        <v>0</v>
-      </c>
-      <c r="F86">
+      <c r="D87">
+        <v>1</v>
+      </c>
+      <c r="E87">
+        <v>0</v>
+      </c>
+      <c r="F87">
         <v>49</v>
       </c>
-      <c r="G86">
+      <c r="G87">
         <v>50</v>
       </c>
-      <c r="H86">
+      <c r="H87">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>78</v>
+      </c>
+      <c r="B88">
+        <v>1</v>
+      </c>
+      <c r="C88" t="s">
+        <v>79</v>
+      </c>
+      <c r="D88">
+        <v>1</v>
+      </c>
+      <c r="E88">
+        <v>0</v>
+      </c>
+      <c r="F88">
+        <v>64</v>
+      </c>
+      <c r="G88">
+        <v>65</v>
+      </c>
+      <c r="H88">
         <v>99</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H86" xr:uid="{EB6437B3-F8C6-4C30-BAA1-BB8B4D93E54D}"/>
+  <autoFilter ref="A1:H87" xr:uid="{EB6437B3-F8C6-4C30-BAA1-BB8B4D93E54D}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added four new metric/package types for trade up teams to consider when selecting package to offer
</commit_message>
<xml_diff>
--- a/Files/TestFiles/PositionNeeds.xlsx
+++ b/Files/TestFiles/PositionNeeds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Git/MaddenDraftTool/Files/TestFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="492" documentId="8_{7C439BFB-0DBF-4097-AD0B-C529E75DCE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB675B41-063F-4415-8090-19503883423C}"/>
+  <xr:revisionPtr revIDLastSave="494" documentId="8_{7C439BFB-0DBF-4097-AD0B-C529E75DCE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C65CA140-5321-4FE5-95AB-FC69B72DD11B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE15C3C6-B90C-4AA8-AF55-EC28F49C3043}"/>
   </bookViews>
@@ -2235,7 +2235,7 @@
         <v>40</v>
       </c>
       <c r="D80">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E80">
         <v>0</v>
@@ -2255,7 +2255,7 @@
         <v>41</v>
       </c>
       <c r="D81">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="E81">
         <v>0</v>

</xml_diff>

<commit_message>
Added team need filtering to UI to only show team needs of the current round and next round
</commit_message>
<xml_diff>
--- a/Files/TestFiles/PositionNeeds.xlsx
+++ b/Files/TestFiles/PositionNeeds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Git/MaddenDraftTool/Files/TestFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="494" documentId="8_{7C439BFB-0DBF-4097-AD0B-C529E75DCE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C65CA140-5321-4FE5-95AB-FC69B72DD11B}"/>
+  <xr:revisionPtr revIDLastSave="496" documentId="8_{7C439BFB-0DBF-4097-AD0B-C529E75DCE6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03586873-364B-4F00-A6C0-D3A20B73E24E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE15C3C6-B90C-4AA8-AF55-EC28F49C3043}"/>
   </bookViews>
@@ -2275,7 +2275,7 @@
         <v>17</v>
       </c>
       <c r="D82">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E82">
         <v>0</v>
@@ -2295,7 +2295,7 @@
         <v>50</v>
       </c>
       <c r="D83">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E83">
         <v>0</v>

</xml_diff>

<commit_message>
Add trade-up covet multiplier and GM trait influence on M_up, small tweaks to trade chances
</commit_message>
<xml_diff>
--- a/Files/TestFiles/PositionNeeds.xlsx
+++ b/Files/TestFiles/PositionNeeds.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ethpe\OneDrive\Documents\Git\MaddenDraftTool\Files\TestFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Git/MaddenDraftTool/Files/TestFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FAA4E12-0FD1-466C-BAB5-B80840A97439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{5FAA4E12-0FD1-466C-BAB5-B80840A97439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53800490-506D-4882-9119-CCC952B5A767}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE15C3C6-B90C-4AA8-AF55-EC28F49C3043}"/>
   </bookViews>
@@ -1505,7 +1505,7 @@
         <v>59</v>
       </c>
       <c r="D31">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E31">
         <v>73</v>
@@ -1515,11 +1515,11 @@
       </c>
       <c r="G31">
         <f t="shared" si="0"/>
-        <v>1.875</v>
+        <v>2.25</v>
       </c>
       <c r="H31">
         <f t="shared" si="1"/>
-        <v>3.125</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1561,7 +1561,7 @@
         <v>60</v>
       </c>
       <c r="D33">
-        <v>2.25</v>
+        <v>2.75</v>
       </c>
       <c r="E33">
         <v>70</v>
@@ -1571,11 +1571,11 @@
       </c>
       <c r="G33">
         <f t="shared" si="0"/>
-        <v>1.6875</v>
+        <v>2.0625</v>
       </c>
       <c r="H33">
         <f t="shared" si="1"/>
-        <v>2.8125</v>
+        <v>3.4375</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -1953,7 +1953,7 @@
         <v>54</v>
       </c>
       <c r="D47">
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="E47">
         <v>75</v>
@@ -1963,11 +1963,11 @@
       </c>
       <c r="G47">
         <f t="shared" si="0"/>
-        <v>1.6875</v>
+        <v>1.875</v>
       </c>
       <c r="H47">
         <f t="shared" si="1"/>
-        <v>2.8125</v>
+        <v>3.125</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -2009,7 +2009,7 @@
         <v>55</v>
       </c>
       <c r="D49">
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="E49">
         <v>74</v>
@@ -2019,11 +2019,11 @@
       </c>
       <c r="G49">
         <f t="shared" si="0"/>
-        <v>1.6875</v>
+        <v>1.875</v>
       </c>
       <c r="H49">
         <f t="shared" si="1"/>
-        <v>2.8125</v>
+        <v>3.125</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sim pick tuning, prospect type tiers, round modifier adjustments
</commit_message>
<xml_diff>
--- a/Files/TestFiles/PositionNeeds.xlsx
+++ b/Files/TestFiles/PositionNeeds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Git/MaddenDraftTool/Files/TestFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{5FAA4E12-0FD1-466C-BAB5-B80840A97439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53800490-506D-4882-9119-CCC952B5A767}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{5FAA4E12-0FD1-466C-BAB5-B80840A97439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{337A1328-E6C6-4C29-A3EB-625E9A238F7F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE15C3C6-B90C-4AA8-AF55-EC28F49C3043}"/>
   </bookViews>
@@ -329,6 +329,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1001,7 +1005,7 @@
         <v>21</v>
       </c>
       <c r="D13">
-        <v>3</v>
+        <v>3.25</v>
       </c>
       <c r="E13">
         <v>75</v>
@@ -1011,11 +1015,11 @@
       </c>
       <c r="G13">
         <f t="shared" si="0"/>
-        <v>2.25</v>
+        <v>2.4375</v>
       </c>
       <c r="H13">
         <f t="shared" si="1"/>
-        <v>3.75</v>
+        <v>4.0625</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1141,7 +1145,7 @@
         <v>23</v>
       </c>
       <c r="D18">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -1151,11 +1155,11 @@
       </c>
       <c r="G18">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>1.6875</v>
       </c>
       <c r="H18">
         <f t="shared" si="1"/>
-        <v>2.5</v>
+        <v>2.8125</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -1169,7 +1173,7 @@
         <v>23</v>
       </c>
       <c r="D19">
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="E19">
         <v>70</v>
@@ -1179,11 +1183,11 @@
       </c>
       <c r="G19">
         <f t="shared" si="0"/>
-        <v>1.3125</v>
+        <v>1.5</v>
       </c>
       <c r="H19">
         <f t="shared" si="1"/>
-        <v>2.1875</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -1225,7 +1229,7 @@
         <v>24</v>
       </c>
       <c r="D21">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -1235,11 +1239,11 @@
       </c>
       <c r="G21">
         <f t="shared" si="0"/>
-        <v>0.9375</v>
+        <v>1.125</v>
       </c>
       <c r="H21">
         <f t="shared" si="1"/>
-        <v>1.5625</v>
+        <v>1.875</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -1561,7 +1565,7 @@
         <v>60</v>
       </c>
       <c r="D33">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="E33">
         <v>70</v>
@@ -1571,11 +1575,11 @@
       </c>
       <c r="G33">
         <f t="shared" si="0"/>
-        <v>2.0625</v>
+        <v>2.25</v>
       </c>
       <c r="H33">
         <f t="shared" si="1"/>
-        <v>3.4375</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -1953,7 +1957,7 @@
         <v>54</v>
       </c>
       <c r="D47">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="E47">
         <v>75</v>
@@ -1963,11 +1967,11 @@
       </c>
       <c r="G47">
         <f t="shared" si="0"/>
-        <v>1.875</v>
+        <v>2.0625</v>
       </c>
       <c r="H47">
         <f t="shared" si="1"/>
-        <v>3.125</v>
+        <v>3.4375</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -2569,7 +2573,7 @@
         <v>32</v>
       </c>
       <c r="D69">
-        <v>3</v>
+        <v>3.25</v>
       </c>
       <c r="E69">
         <v>75</v>
@@ -2579,11 +2583,11 @@
       </c>
       <c r="G69">
         <f t="shared" si="14"/>
-        <v>2.25</v>
+        <v>2.4375</v>
       </c>
       <c r="H69">
         <f t="shared" si="15"/>
-        <v>3.75</v>
+        <v>4.0625</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
@@ -2709,7 +2713,7 @@
         <v>34</v>
       </c>
       <c r="D74">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="E74">
         <v>0</v>
@@ -2719,11 +2723,11 @@
       </c>
       <c r="G74">
         <f t="shared" si="14"/>
-        <v>1.5</v>
+        <v>1.6875</v>
       </c>
       <c r="H74">
         <f t="shared" si="15"/>
-        <v>2.5</v>
+        <v>2.8125</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
@@ -2737,7 +2741,7 @@
         <v>34</v>
       </c>
       <c r="D75">
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="E75">
         <v>70</v>
@@ -2747,11 +2751,11 @@
       </c>
       <c r="G75">
         <f t="shared" si="14"/>
-        <v>1.3125</v>
+        <v>1.5</v>
       </c>
       <c r="H75">
         <f t="shared" si="15"/>
-        <v>2.1875</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
@@ -2793,7 +2797,7 @@
         <v>35</v>
       </c>
       <c r="D77">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="E77">
         <v>0</v>
@@ -2803,11 +2807,11 @@
       </c>
       <c r="G77">
         <f t="shared" si="14"/>
-        <v>0.9375</v>
+        <v>1.125</v>
       </c>
       <c r="H77">
         <f t="shared" si="15"/>
-        <v>1.5625</v>
+        <v>1.875</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add Non-Premium R1 trait, sim report modal, and BPA/need tracking
</commit_message>
<xml_diff>
--- a/Files/TestFiles/PositionNeeds.xlsx
+++ b/Files/TestFiles/PositionNeeds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Git/MaddenDraftTool/Files/TestFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{5FAA4E12-0FD1-466C-BAB5-B80840A97439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{337A1328-E6C6-4C29-A3EB-625E9A238F7F}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{5FAA4E12-0FD1-466C-BAB5-B80840A97439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61394B5F-51FF-4173-AA70-645DFD2E5185}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE15C3C6-B90C-4AA8-AF55-EC28F49C3043}"/>
   </bookViews>
@@ -1733,7 +1733,7 @@
         <v>64</v>
       </c>
       <c r="D39">
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="E39">
         <v>70</v>
@@ -1743,11 +1743,11 @@
       </c>
       <c r="G39">
         <f t="shared" si="0"/>
-        <v>1.6875</v>
+        <v>1.875</v>
       </c>
       <c r="H39">
         <f t="shared" si="1"/>
-        <v>2.8125</v>
+        <v>3.125</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
@@ -1817,7 +1817,7 @@
         <v>27</v>
       </c>
       <c r="D42">
-        <v>3</v>
+        <v>3.25</v>
       </c>
       <c r="E42">
         <v>0</v>
@@ -1827,11 +1827,11 @@
       </c>
       <c r="G42">
         <f t="shared" si="0"/>
-        <v>2.25</v>
+        <v>2.4375</v>
       </c>
       <c r="H42">
         <f t="shared" si="1"/>
-        <v>3.75</v>
+        <v>4.0625</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -1845,7 +1845,7 @@
         <v>27</v>
       </c>
       <c r="D43">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="E43">
         <v>70</v>
@@ -1855,11 +1855,11 @@
       </c>
       <c r="G43">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>1.6875</v>
       </c>
       <c r="H43">
         <f t="shared" si="1"/>
-        <v>2.5</v>
+        <v>2.8125</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -1873,7 +1873,7 @@
         <v>28</v>
       </c>
       <c r="D44">
-        <v>1.5</v>
+        <v>1.75</v>
       </c>
       <c r="E44">
         <v>0</v>
@@ -1883,11 +1883,11 @@
       </c>
       <c r="G44">
         <f t="shared" si="0"/>
-        <v>1.125</v>
+        <v>1.3125</v>
       </c>
       <c r="H44">
         <f t="shared" si="1"/>
-        <v>1.875</v>
+        <v>2.1875</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -1957,7 +1957,7 @@
         <v>54</v>
       </c>
       <c r="D47">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="E47">
         <v>75</v>
@@ -1967,11 +1967,11 @@
       </c>
       <c r="G47">
         <f t="shared" si="0"/>
-        <v>2.0625</v>
+        <v>2.25</v>
       </c>
       <c r="H47">
         <f t="shared" si="1"/>
-        <v>3.4375</v>
+        <v>3.75</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -2013,7 +2013,7 @@
         <v>55</v>
       </c>
       <c r="D49">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="E49">
         <v>74</v>
@@ -2023,11 +2023,11 @@
       </c>
       <c r="G49">
         <f t="shared" si="0"/>
-        <v>1.875</v>
+        <v>2.0625</v>
       </c>
       <c r="H49">
         <f t="shared" si="1"/>
-        <v>3.125</v>
+        <v>3.4375</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
@@ -2041,7 +2041,7 @@
         <v>66</v>
       </c>
       <c r="D50">
-        <v>2</v>
+        <v>2.75</v>
       </c>
       <c r="E50">
         <v>0</v>
@@ -2051,11 +2051,11 @@
       </c>
       <c r="G50">
         <f t="shared" si="0"/>
-        <v>1.5</v>
+        <v>2.0625</v>
       </c>
       <c r="H50">
         <f t="shared" si="1"/>
-        <v>2.5</v>
+        <v>3.4375</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -2069,7 +2069,7 @@
         <v>66</v>
       </c>
       <c r="D51">
-        <v>1.25</v>
+        <v>1.75</v>
       </c>
       <c r="E51">
         <v>70</v>
@@ -2079,11 +2079,11 @@
       </c>
       <c r="G51">
         <f t="shared" si="0"/>
-        <v>0.9375</v>
+        <v>1.3125</v>
       </c>
       <c r="H51">
         <f t="shared" si="1"/>
-        <v>1.5625</v>
+        <v>2.1875</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
@@ -2097,7 +2097,7 @@
         <v>67</v>
       </c>
       <c r="D52">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="E52">
         <v>0</v>
@@ -2107,11 +2107,11 @@
       </c>
       <c r="G52">
         <f t="shared" si="0"/>
-        <v>0.75</v>
+        <v>0.9375</v>
       </c>
       <c r="H52">
         <f t="shared" si="1"/>
-        <v>1.25</v>
+        <v>1.5625</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Shorten round 2 need reach limit, small adjustments to position needs
</commit_message>
<xml_diff>
--- a/Files/TestFiles/PositionNeeds.xlsx
+++ b/Files/TestFiles/PositionNeeds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Git/MaddenDraftTool/Files/TestFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{5FAA4E12-0FD1-466C-BAB5-B80840A97439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61394B5F-51FF-4173-AA70-645DFD2E5185}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{5FAA4E12-0FD1-466C-BAB5-B80840A97439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0503E3B-65DF-4B68-8C34-1C7E2AAA9E32}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE15C3C6-B90C-4AA8-AF55-EC28F49C3043}"/>
   </bookViews>
@@ -725,7 +725,7 @@
         <v>48</v>
       </c>
       <c r="D3">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="E3">
         <v>70</v>
@@ -735,11 +735,11 @@
       </c>
       <c r="G3">
         <f t="shared" ref="G3:G67" si="0">D3-(D3*0.25)</f>
-        <v>1.875</v>
+        <v>2.0625</v>
       </c>
       <c r="H3">
         <f t="shared" ref="H3:H67" si="1">D3+(D3*0.25)</f>
-        <v>3.125</v>
+        <v>3.4375</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -781,7 +781,7 @@
         <v>18</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="E5">
         <v>60</v>
@@ -791,11 +791,11 @@
       </c>
       <c r="G5">
         <f t="shared" si="0"/>
-        <v>0.75</v>
+        <v>0.9375</v>
       </c>
       <c r="H5">
         <f t="shared" si="1"/>
-        <v>1.25</v>
+        <v>1.5625</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -921,7 +921,7 @@
         <v>45</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -931,11 +931,11 @@
       </c>
       <c r="G10">
         <f t="shared" si="0"/>
-        <v>0.75</v>
+        <v>0.9375</v>
       </c>
       <c r="H10">
         <f t="shared" si="1"/>
-        <v>1.25</v>
+        <v>1.5625</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -949,7 +949,7 @@
         <v>45</v>
       </c>
       <c r="D11">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="E11">
         <v>65</v>
@@ -959,11 +959,11 @@
       </c>
       <c r="G11">
         <f t="shared" ref="G11" si="2">D11-(D11*0.25)</f>
-        <v>0.9375</v>
+        <v>0.75</v>
       </c>
       <c r="H11">
         <f t="shared" ref="H11" si="3">D11+(D11*0.25)</f>
-        <v>1.5625</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>